<commit_message>
Articles pushed as of 28th Feb
</commit_message>
<xml_diff>
--- a/TS Jatai Working/prAtiSAkyam Rules Sethu.xlsx
+++ b/TS Jatai Working/prAtiSAkyam Rules Sethu.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\texts\TS Jatai Working\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Github\texts\TS Jatai Working\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8CC9F8D-2ACE-4162-9A40-D62F2C82253C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E30453C-6F20-4EA5-AC97-317987DBD5B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Vowel Elongation" sheetId="1" r:id="rId1"/>
@@ -31,9 +31,10 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>

</xml_diff>

<commit_message>
Visarga sandhi article final
</commit_message>
<xml_diff>
--- a/TS Jatai Working/prAtiSAkyam Rules Sethu.xlsx
+++ b/TS Jatai Working/prAtiSAkyam Rules Sethu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Github\texts\TS Jatai Working\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E30453C-6F20-4EA5-AC97-317987DBD5B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7588B1E2-0295-4BE0-AF24-BE8F430134F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6811,7 +6811,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -6931,6 +6931,7 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -19509,7 +19510,7 @@
       <c r="J49" s="4" t="s">
         <v>1563</v>
       </c>
-      <c r="O49" s="4" t="s">
+      <c r="O49" s="81" t="s">
         <v>1564</v>
       </c>
     </row>
@@ -20260,13 +20261,13 @@
       <c r="K89" s="4" t="s">
         <v>1384</v>
       </c>
-      <c r="L89" s="4" t="s">
+      <c r="L89" s="81" t="s">
         <v>557</v>
       </c>
       <c r="M89" s="4" t="s">
         <v>1958</v>
       </c>
-      <c r="N89" s="4" t="s">
+      <c r="N89" s="81" t="s">
         <v>1959</v>
       </c>
     </row>
@@ -20305,7 +20306,7 @@
       <c r="M91" s="4" t="s">
         <v>1960</v>
       </c>
-      <c r="N91" s="4" t="s">
+      <c r="N91" s="81" t="s">
         <v>1961</v>
       </c>
     </row>
@@ -20396,7 +20397,7 @@
       <c r="H97" s="4" t="s">
         <v>1970</v>
       </c>
-      <c r="J97" s="4" t="s">
+      <c r="J97" s="81" t="s">
         <v>1546</v>
       </c>
     </row>
@@ -20447,7 +20448,7 @@
       </c>
     </row>
     <row r="100" spans="1:15" s="4" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="C100" s="4" t="s">
+      <c r="C100" s="81" t="s">
         <v>1976</v>
       </c>
       <c r="F100" s="5" t="s">
@@ -20479,7 +20480,7 @@
       <c r="G101" s="4" t="s">
         <v>1979</v>
       </c>
-      <c r="K101" s="4" t="s">
+      <c r="K101" s="81" t="s">
         <v>1979</v>
       </c>
       <c r="L101" s="4" t="s">

</xml_diff>